<commit_message>
Updated for EA 23.237 Stable. Added an experimental optimization option to reduce lag when gaining massive EXP. This feature is not vanilla and may discard some leftover EXP.
EA 23.237 Stable に対応しました。大量の経験値取得時のラグを軽減するための実験的な最適化オプションを追加しました。この機能はバニラとは異なる挙動となり、一部の残り経験値が失われる場合があります。

现已更新至 EA 23.237 稳定版 新增实验性优化选项 在大量经验获取时减少卡顿 此功能与原版行为不同 并可能损失少量剩余经验值
</commit_message>
<xml_diff>
--- a/translations.xlsx
+++ b/translations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -101,6 +101,33 @@
 启用后，升级后剩余经验值将除以2。
 禁用后，所有经验值将被完全保留。
 需要重启游戏才能生效。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toggle02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enable Optimization (Experimental)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">最適化を有効化（実験的）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">启用优化（实验性）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tooltip02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When enabled, extra levels from massive EXP gains are optimized and processed differently from vanilla behavior.
+This can significantly reduce lag when gaining very large EXP amounts, but some leftover EXP will be lost during processing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有効にすると、大量の経験値を一度に獲得した際に、追加のレベルアップ処理が最適化され、バニラとは異なる挙動になります。
+ラグを大幅に軽減できますが、一部の残り経験値が処理中に失われる場合があります。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">启用后，大量经验一次性获取时会使用优化的升级处理方式，与原版行为不同。
+可以显著减少卡顿，不过在此过程中可能会损失少量剩余经验值。</t>
   </si>
 </sst>
 </file>
@@ -110,7 +137,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -137,6 +164,11 @@
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Noto Sans SC"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -181,7 +213,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -195,6 +227,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -321,8 +357,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="65.95"/>
@@ -415,6 +451,34 @@
         <v>23</v>
       </c>
     </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Fixed the diminishing returns (DR) calculation during level ups. As a result, very large EXP gains may now grant fewer levels than before. The Optimization setting has also been updated to simulate perfect +1000 EXP per level behavior by processing each level threshold individually, which reduces lag when handling massive EXP gains.
</commit_message>
<xml_diff>
--- a/translations.xlsx
+++ b/translations.xlsx
@@ -118,16 +118,16 @@
     <t xml:space="preserve">tooltip02</t>
   </si>
   <si>
-    <t xml:space="preserve">When enabled, extra levels from massive EXP gains are optimized and processed differently from vanilla behavior.
-This can significantly reduce lag when gaining very large EXP amounts, but some leftover EXP will be lost during processing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">有効にすると、大量の経験値を一度に獲得した際に、追加のレベルアップ処理が最適化され、バニラとは異なる挙動になります。
-ラグを大幅に軽減できますが、一部の残り経験値が処理中に失われる場合があります。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">启用后，大量经验一次性获取时会使用优化的升级处理方式，与原版行为不同。
-可以显著减少卡顿，不过在此过程中可能会损失少量剩余经验值。</t>
+    <t xml:space="preserve">When enabled, large EXP gains are processed using an optimized batch-leveling method.
+This produces results close to leveling one step at a time while greatly reducing lag during massive EXP gains.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有効にすると、大量の経験値獲得を段階的に処理する最適化方式が適用されます。
+手動で1レベルずつ上げる場合に近い結果となり、処理の重さを大幅に軽減できます。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">启用后，大量经验将按逐级最佳方式进行优化处理。
+结果接近手动逐级升级，并可显著减轻卡顿。</t>
   </si>
 </sst>
 </file>
@@ -169,6 +169,7 @@
       <sz val="10"/>
       <name val="Noto Sans SC"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">

</xml_diff>